<commit_message>
Complete the sourcing audit: every remaining input dispositioned
Reverse-engineered the workbook's own patterns to resolve more of the
"unsourced" set: EqEarn = Peq/PeRatio exactly (0.000% over 82 quarters,
wired as a post-merge derivation); GovDebt = linear interpolation between
June-quarter annual net debt levels (validated exactly, +26.9/quarter
Jun-2023 to Jun-2024); GovDef = quarterly interpolation of annual
general-government net lending (annual sums identified); PcpiExGst = a
genuinely separate AEM splice (ratio to Pcpi drifts); Ustar = unused by
the model (superseded by LurHpf). PeRatio's free-endpoint search is
exhausted with evidence recorded (ASX archive index/market-cap only,
marketindex Cloudflare-gated, RBA tables discontinued 2011) - it remains
the LSEG channel, and EqEarn now follows automatically once it extends.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/Data.xlsx
+++ b/data-raw/Data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="8" state="visible" r:id="rId3"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="634">
   <si>
     <t>date</t>
   </si>
@@ -1907,6 +1907,21 @@
   <si>
     <t xml:space="preserve">Public-sector net debt from annual fiscal data (ABS GFS annual net debt checked: 846.6b 2023-24, 954.9b 2024-25; the workbook's quarterly path is a custom interpolation - the derivation is needed)</t>
   </si>
+  <si>
+    <t xml:space="preserve">Derived: Peq / PeRatio (validated 0.000% over 82 quarters; the model's EqYield identity). PeRatio upstream is the LSEG/Refinitiv ASX calculated P/E - free endpoints tested (ASX archive: index/market-cap only; marketindex.com.au: Cloudflare; RBA: discontinued 2011; Yahoo/FRED: no P/E)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custom quarterly interpolation of the annual fiscal balance (structure identified: annual sums match general-government net lending, e.g. 2022: ~80.6b, 2023: ~28.2b, 2024: ~45.8b; GFS quarterly checked and differs - the owner's interpolation kernel and annual vintage are needed to extend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linear interpolation between June-quarter annual net debt levels (structure validated exactly: +26.9/quarter Jun-2023 to Jun-2024 = 661.7 to 769.3; current GFS annual net debt 783.8/846.6/954.9 does not match the workbook's vintage - the owner's annual source is needed to extend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AEM PCPIUX internal splice (CPI excluding GST effects) - not reproducible from published ABS series (ratio to Pcpi drifts 0.0095-0.0102); the splice is the source record</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legacy EViews SEM NAIRU estimate via Masterdata - unused by the model (superseded by LurHpf per the variable audit); kept for history</t>
+  </si>
 </sst>
 </file>
 
@@ -3565,7 +3580,7 @@
         <v>218</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="D95" s="2" t="s">
         <v>71</v>
@@ -3747,7 +3762,7 @@
         <v>460</v>
       </c>
       <c r="C108" s="2" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="D108" s="2" t="s">
         <v>244</v>
@@ -3761,7 +3776,7 @@
         <v>462</v>
       </c>
       <c r="C109" s="2" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="D109" s="2" t="s">
         <v>220</v>
@@ -3869,7 +3884,7 @@
         <v>233</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>234</v>
+        <v>633</v>
       </c>
       <c r="D117" s="2" t="s">
         <v>329</v>
@@ -3911,7 +3926,7 @@
         <v>241</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>242</v>
+        <v>632</v>
       </c>
       <c r="D120" s="2" t="s">
         <v>243</v>
@@ -45970,7 +45985,7 @@
         <v>16.2143333333333</v>
       </c>
       <c r="CQ124" t="n">
-        <v>252.899697798244</v>
+        <v>252.899697798245</v>
       </c>
       <c r="CR124" t="n">
         <v>47.1</v>
@@ -47448,7 +47463,7 @@
         <v>15.8187301587302</v>
       </c>
       <c r="CQ128" t="n">
-        <v>321.593449597624</v>
+        <v>321.593449597623</v>
       </c>
       <c r="CR128" t="n">
         <v>53.2</v>
@@ -47819,7 +47834,7 @@
         <v>14.8493442622951</v>
       </c>
       <c r="CQ129" t="n">
-        <v>339.004868570672</v>
+        <v>339.004868570671</v>
       </c>
       <c r="CR129" t="n">
         <v>21.4</v>
@@ -48561,7 +48576,7 @@
         <v>15.4328571428571</v>
       </c>
       <c r="CQ131" t="n">
-        <v>365.7326668518</v>
+        <v>365.732666851801</v>
       </c>
       <c r="CR131" t="n">
         <v>50.6</v>
@@ -48932,7 +48947,7 @@
         <v>14.8138095238095</v>
       </c>
       <c r="CQ132" t="n">
-        <v>403.596386897682</v>
+        <v>403.596386897683</v>
       </c>
       <c r="CR132" t="n">
         <v>76</v>
@@ -49303,7 +49318,7 @@
         <v>15.1886885245902</v>
       </c>
       <c r="CQ133" t="n">
-        <v>415.480243062676</v>
+        <v>415.480243062675</v>
       </c>
       <c r="CR133" t="n">
         <v>49.2</v>
@@ -50787,7 +50802,7 @@
         <v>13.3449206349206</v>
       </c>
       <c r="CQ137" t="n">
-        <v>399.620211007101</v>
+        <v>399.620211007102</v>
       </c>
       <c r="CR137" t="n">
         <v>65.1</v>
@@ -51158,7 +51173,7 @@
         <v>12.3561538461539</v>
       </c>
       <c r="CQ138" t="n">
-        <v>374.817281952313</v>
+        <v>374.817281952311</v>
       </c>
       <c r="CR138" t="n">
         <v>84.1</v>
@@ -52642,7 +52657,7 @@
         <v>11.6742424242424</v>
       </c>
       <c r="CQ142" t="n">
-        <v>405.962102530824</v>
+        <v>405.962102530825</v>
       </c>
       <c r="CR142" t="n">
         <v>62.5</v>
@@ -53755,7 +53770,7 @@
         <v>16.8435849056604</v>
       </c>
       <c r="CQ145" t="n">
-        <v>256.762442450516</v>
+        <v>256.762442450515</v>
       </c>
       <c r="CR145" t="n">
         <v>32</v>
@@ -54868,7 +54883,7 @@
         <v>15.3264516129032</v>
       </c>
       <c r="CQ148" t="n">
-        <v>321.574760060616</v>
+        <v>321.574760060617</v>
       </c>
       <c r="CR148" t="n">
         <v>61</v>
@@ -56352,7 +56367,7 @@
         <v>12.3142857142857</v>
       </c>
       <c r="CQ152" t="n">
-        <v>358.932714617169</v>
+        <v>358.93271461717</v>
       </c>
       <c r="CR152" t="n">
         <v>74</v>
@@ -56723,7 +56738,7 @@
         <v>12.4459016393443</v>
       </c>
       <c r="CQ153" t="n">
-        <v>332.278055848261</v>
+        <v>332.27805584826</v>
       </c>
       <c r="CR153" t="n">
         <v>51.9</v>
@@ -58578,7 +58593,7 @@
         <v>16.6713636363636</v>
       </c>
       <c r="CQ158" t="n">
-        <v>312.973798293208</v>
+        <v>312.973798293209</v>
       </c>
       <c r="CR158" t="n">
         <v>54.2</v>
@@ -59320,7 +59335,7 @@
         <v>16.086935483871</v>
       </c>
       <c r="CQ160" t="n">
-        <v>335.862601389627</v>
+        <v>335.862601389626</v>
       </c>
       <c r="CR160" t="n">
         <v>65</v>
@@ -59691,7 +59706,7 @@
         <v>15.7631147540984</v>
       </c>
       <c r="CQ161" t="n">
-        <v>341.429982840206</v>
+        <v>341.429982840205</v>
       </c>
       <c r="CR161" t="n">
         <v>30.4</v>
@@ -60804,7 +60819,7 @@
         <v>14.3554838709677</v>
       </c>
       <c r="CQ164" t="n">
-        <v>408.338726349378</v>
+        <v>408.338726349379</v>
       </c>
       <c r="CR164" t="n">
         <v>63.8</v>
@@ -61175,7 +61190,7 @@
         <v>14.5253225806452</v>
       </c>
       <c r="CQ165" t="n">
-        <v>375.289427806833</v>
+        <v>375.289427806832</v>
       </c>
       <c r="CR165" t="n">
         <v>33.3</v>
@@ -61546,7 +61561,7 @@
         <v>14.4622727272727</v>
       </c>
       <c r="CQ166" t="n">
-        <v>349.779048936103</v>
+        <v>349.779048936104</v>
       </c>
       <c r="CR166" t="n">
         <v>50.4</v>
@@ -62288,7 +62303,7 @@
         <v>14.7988333333333</v>
       </c>
       <c r="CQ168" t="n">
-        <v>348.122036647033</v>
+        <v>348.122036647034</v>
       </c>
       <c r="CR168" t="n">
         <v>73</v>
@@ -62659,7 +62674,7 @@
         <v>15.7544444444445</v>
       </c>
       <c r="CQ169" t="n">
-        <v>337.073136328373</v>
+        <v>337.073136328372</v>
       </c>
       <c r="CR169" t="n">
         <v>43.6</v>
@@ -63030,7 +63045,7 @@
         <v>16.7315151515152</v>
       </c>
       <c r="CQ170" t="n">
-        <v>330.227116311081</v>
+        <v>330.22711631108</v>
       </c>
       <c r="CR170" t="n">
         <v>73.7</v>
@@ -63772,7 +63787,7 @@
         <v>17.9634920634921</v>
       </c>
       <c r="CQ172" t="n">
-        <v>328.655474065565</v>
+        <v>328.655474065564</v>
       </c>
       <c r="CR172" t="n">
         <v>88.8</v>
@@ -64143,7 +64158,7 @@
         <v>17.6606557377049</v>
       </c>
       <c r="CQ173" t="n">
-        <v>326.37519725239</v>
+        <v>326.375197252391</v>
       </c>
       <c r="CR173" t="n">
         <v>47.3</v>
@@ -64514,7 +64529,7 @@
         <v>16.3112307692308</v>
       </c>
       <c r="CQ174" t="n">
-        <v>352.205181894495</v>
+        <v>352.205181894494</v>
       </c>
       <c r="CR174" t="n">
         <v>69.7</v>
@@ -65256,7 +65271,7 @@
         <v>15.7241935483871</v>
       </c>
       <c r="CQ176" t="n">
-        <v>373.240127192533</v>
+        <v>373.240127192532</v>
       </c>
       <c r="CR176" t="n">
         <v>85.1</v>
@@ -65627,7 +65642,7 @@
         <v>15.8003225806452</v>
       </c>
       <c r="CQ177" t="n">
-        <v>398.074151201486</v>
+        <v>398.074151201485</v>
       </c>
       <c r="CR177" t="n">
         <v>47.6</v>
@@ -66740,7 +66755,7 @@
         <v>12.6023728813559</v>
       </c>
       <c r="CQ180" t="n">
-        <v>496.866745568497</v>
+        <v>496.866745568498</v>
       </c>
       <c r="CR180" t="n">
         <v>83.6</v>
@@ -67111,7 +67126,7 @@
         <v>14.3034426229508</v>
       </c>
       <c r="CQ181" t="n">
-        <v>468.362769481152</v>
+        <v>468.362769481153</v>
       </c>
       <c r="CR181" t="n">
         <v>38.2</v>
@@ -68595,7 +68610,7 @@
         <v>15.1154838709677</v>
       </c>
       <c r="CQ185" t="n">
-        <v>397.029962866533</v>
+        <v>397.029962866534</v>
       </c>
       <c r="CR185" t="n">
         <v>-8.3</v>
@@ -69708,7 +69723,7 @@
         <v>21.4329508196721</v>
       </c>
       <c r="CQ188" t="n">
-        <v>327.393090155345</v>
+        <v>327.393090155346</v>
       </c>
       <c r="CR188" t="n">
         <v>-14.2</v>
@@ -70079,7 +70094,7 @@
         <v>21.3114516129032</v>
       </c>
       <c r="CQ189" t="n">
-        <v>355.911935881814</v>
+        <v>355.911935881815</v>
       </c>
       <c r="CR189" t="n">
         <v>1.1</v>
@@ -71192,7 +71207,7 @@
         <v>13.8409836065574</v>
       </c>
       <c r="CQ192" t="n">
-        <v>562.792372379486</v>
+        <v>562.792372379485</v>
       </c>
       <c r="CR192" t="n">
         <v>107.5</v>
@@ -71563,7 +71578,7 @@
         <v>10.9762295081967</v>
       </c>
       <c r="CQ193" t="n">
-        <v>614.646404301396</v>
+        <v>614.646404301398</v>
       </c>
       <c r="CR193" t="n">
         <v>78</v>
@@ -71934,7 +71949,7 @@
         <v>10.3707692307692</v>
       </c>
       <c r="CQ194" t="n">
-        <v>643.992731048806</v>
+        <v>643.992731048808</v>
       </c>
       <c r="CR194" t="n">
         <v>127.7</v>
@@ -72305,7 +72320,7 @@
         <v>10.7598387096774</v>
       </c>
       <c r="CQ195" t="n">
-        <v>671.171770772436</v>
+        <v>671.171770772438</v>
       </c>
       <c r="CR195" t="n">
         <v>124.6</v>
@@ -72676,7 +72691,7 @@
         <v>11.4987301587302</v>
       </c>
       <c r="CQ196" t="n">
-        <v>641.227326688937</v>
+        <v>641.227326688935</v>
       </c>
       <c r="CR196" t="n">
         <v>165.5</v>
@@ -73047,7 +73062,7 @@
         <v>11.3130508474576</v>
       </c>
       <c r="CQ197" t="n">
-        <v>654.244385515454</v>
+        <v>654.244385515456</v>
       </c>
       <c r="CR197" t="n">
         <v>120.5</v>
@@ -74160,7 +74175,7 @@
         <v>17.2203333333333</v>
       </c>
       <c r="CQ200" t="n">
-        <v>473.492576605176</v>
+        <v>473.492576605177</v>
       </c>
       <c r="CR200" t="n">
         <v>128.7</v>
@@ -74531,7 +74546,7 @@
         <v>20.1301639344262</v>
       </c>
       <c r="CQ201" t="n">
-        <v>398.09909278955</v>
+        <v>398.099092789551</v>
       </c>
       <c r="CR201" t="n">
         <v>55.8</v>
@@ -74902,7 +74917,7 @@
         <v>19.0115151515152</v>
       </c>
       <c r="CQ202" t="n">
-        <v>440.801268768529</v>
+        <v>440.801268768528</v>
       </c>
       <c r="CR202" t="n">
         <v>81.6</v>
@@ -75273,7 +75288,7 @@
         <v>17.4153333333333</v>
       </c>
       <c r="CQ203" t="n">
-        <v>503.209510846212</v>
+        <v>503.209510846213</v>
       </c>
       <c r="CR203" t="n">
         <v>64.3</v>

</xml_diff>